<commit_message>
Over all sub area and loan category remove
</commit_message>
<xml_diff>
--- a/uploads/excel_format/area_creation_format.xlsx
+++ b/uploads/excel_format/area_creation_format.xlsx
@@ -1,13 +1,8 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="153222"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\marudham\uploads\excel_format\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="6" rupBuild="9302"/>
+  <workbookPr/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12435"/>
   </bookViews>
@@ -61,7 +56,7 @@
     <definedName name="VirudhunagarList">#REF!</definedName>
     <definedName name="YanamList">#REF!</definedName>
   </definedNames>
-  <calcPr calcId="152511"/>
+  <calcPr calcId="144525"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -71,7 +66,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
   <si>
     <t>State</t>
   </si>
@@ -83,9 +78,6 @@
   </si>
   <si>
     <t>Area</t>
-  </si>
-  <si>
-    <t>Sub Area</t>
   </si>
   <si>
     <t>Pincode</t>
@@ -193,7 +185,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:latin typeface="Calibri Light"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -228,7 +220,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -405,7 +397,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -413,18 +405,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:E1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.85546875" customWidth="1"/>
     <col min="2" max="2" width="19" customWidth="1"/>
     <col min="3" max="3" width="19.140625" customWidth="1"/>
     <col min="4" max="4" width="18.42578125" customWidth="1"/>
-    <col min="5" max="5" width="19.140625" customWidth="1"/>
-    <col min="6" max="6" width="18.5703125" customWidth="1"/>
+    <col min="5" max="5" width="18.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -440,9 +431,6 @@
       <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>